<commit_message>
feat(2026-05-23): add training slide, extra Kahoot questions, and cleanup
- Add 'How Are Image Models Trained?' slide (slide 5) to presentation
- Add 2 training-related Kahoot questions (17 total)
- Update Teams posts: digital-only submission to Ishwari ma'am
- Update .gitignore for project needs (Office temp files, IDE, .claude/)
- Remove .claude/settings.local.json from tracking
</commit_message>
<xml_diff>
--- a/2026-05-23_AI_Image_and_Multimodal_Models/2026-05-23_Kahoot_Import.xlsx
+++ b/2026-05-23_AI_Image_and_Multimodal_Models/2026-05-23_Kahoot_Import.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -948,6 +948,72 @@
         <v>2</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>What do AI image models learn from during training?</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>A single artist's sketchbook</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Billions of images paired with text descriptions from the internet</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Only photographs taken by professional cameras</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Screenshots of video games</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>25</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>During training, what does the AI learn to do with noise?</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Add more noise to make images blurry</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Remove noise step by step to recover the original image</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Replace noise with random colors</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Ignore the noise completely</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>25</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(2026-05-30): add building with AI class materials
</commit_message>
<xml_diff>
--- a/2026-05-23_AI_Image_and_Multimodal_Models/2026-05-23_Kahoot_Import.xlsx
+++ b/2026-05-23_AI_Image_and_Multimodal_Models/2026-05-23_Kahoot_Import.xlsx
@@ -565,7 +565,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AI that can understand and generate multiple types of data (text, images, audio)</t>
+          <t>AI that understands and generates multiple data types (text, images, audio)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A golden retriever in a sunflower field, watercolor style, warm sunset lighting</t>
+          <t>A golden retriever in a sunflower field, watercolor style, sunset light</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">

</xml_diff>